<commit_message>
Add g6e.4xlarge upgrade comparison to cost estimate
Section D in the Cost Estimate tab compares the current g5.xlarge (A10G
24GB) against a g6e.4xlarge (L40S 48GB) upgrade: specs, on-demand and
Savings Plan $/mo, deltas, fit, and the GPU-quota prerequisite.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Todozee_Past-Life_AWS_Deployment.xlsx
+++ b/Todozee_Past-Life_AWS_Deployment.xlsx
@@ -1341,15 +1341,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1955,47 +1955,275 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>D.  Upgrade option — g5.xlarge (current)  vs  g6e.4xlarge (NVIDIA L40S)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>g5.xlarge (current)</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>g6e.4xlarge (upgrade)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA A10G, 24 GB</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA L40S, 48 GB</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>2x VRAM; ~2.5-3x FP16 compute</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>vCPU / RAM</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>4 vCPU / 16 GiB</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>16 vCPU / 128 GiB</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>4x vCPU, 8x RAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>On-Demand $/hr</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>1.208</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>3.608</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>~3.0x</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>On-Demand compute $/mo</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>882</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>2,634</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>+1,752 /mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>EC2-Instance SP 1yr No-Up $/mo</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>556</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>1,659</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>+1,104 /mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>EC2-Instance SP 3yr All-Up $/mo</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>990</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>+659 /mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Best suited for</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Model fits in 24 GB (current Gemma 4 E2B ~10 GB) at current load</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Larger models (Gemma 4 12B / 31B), high concurrency, or multi-model serving</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Quota / availability</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Running now</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Needs G-quota bump: 16 vCPU vs 4 free -&gt; raise 24 to 36; offered ap-south-1 AZ a/b</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Recommendation: stay on g5.xlarge — the current model fits the A10G with headroom. Upgrade to g6e.4xlarge only to run a larger Gemma 4 variant or for substantially higher throughput; it roughly triples compute cost and requires a GPU-quota increase first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>- A Savings Plan is an account-wide hourly-spend commitment; it will also automatically discount the other GPU instances (doc-reader, translation) up to the committed amount.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>- Size the commitment to your steady-state 24x7 GPU $/hr baseline, not to one instance, so it keeps applying if you resize.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
         <is>
           <t>- Prices are AWS list prices pulled 2026-06-30; exclude taxes and any private/EDP discounts.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="23">
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="C28:F28"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="D37:F37"/>
     <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="C29:F29"/>
     <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="D36:F36"/>
     <mergeCell ref="C27:F27"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="C28:F28"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>